<commit_message>
Add vegetarian + keto-friendly recipe listings to batch
Extends the recipe-diet-listing template to cover two more diet listing
pages, reusing the existing block/parser/transformer infrastructure.

- page-templates.json: add vegetarian + keto-friendly URLs (3 total)
- urls-recipe-diet-listing-batch2.txt: batch URL list for the two new pages
- bd-snapshots: Bright Data snapshots of both bot-protected sources for
  offline re-import
- reports: per-page import reports + refreshed xlsx

Content .plain.html is intentionally not committed (content/ is gitignored;
Document Authoring is the source of truth — both pages uploaded + published).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-recipe-diet-listing.report.xlsx
+++ b/tools/importer/reports/import-recipe-diet-listing.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="33">
   <si>
     <t>_reportFile</t>
   </si>
@@ -61,18 +61,33 @@
     <t>https://www.albertsons.com/</t>
   </si>
   <si>
+    <t>recipes/diet/keto-friendly.report.json</t>
+  </si>
+  <si>
+    <t>["cards-recipe-grid"]</t>
+  </si>
+  <si>
+    <t>recipes/diet/keto-friendly</t>
+  </si>
+  <si>
+    <t>recipe-diet-listing</t>
+  </si>
+  <si>
+    <t>2026-09-15T16:47:15.103Z</t>
+  </si>
+  <si>
+    <t>Keto-friendly recipes - Shop for keto diet friendly meals | Albertsons</t>
+  </si>
+  <si>
+    <t>https://www.albertsons.com/recipes/diet/keto-friendly</t>
+  </si>
+  <si>
     <t>recipes/diet/pescatarian.report.json</t>
   </si>
   <si>
-    <t>["cards-recipe-grid"]</t>
-  </si>
-  <si>
     <t>recipes/diet/pescatarian</t>
   </si>
   <si>
-    <t>recipe-diet-listing</t>
-  </si>
-  <si>
     <t>2026-09-15T15:16:23.398Z</t>
   </si>
   <si>
@@ -80,6 +95,21 @@
   </si>
   <si>
     <t>https://www.albertsons.com/recipes/diet/pescatarian</t>
+  </si>
+  <si>
+    <t>recipes/diet/vegetarian.report.json</t>
+  </si>
+  <si>
+    <t>recipes/diet/vegetarian</t>
+  </si>
+  <si>
+    <t>2026-09-15T16:47:10.760Z</t>
+  </si>
+  <si>
+    <t>Vegetarian recipes - Shop for easy vegetarian meals | Albertsons</t>
+  </si>
+  <si>
+    <t>https://www.albertsons.com/recipes/diet/vegetarian</t>
   </si>
 </sst>
 </file>
@@ -468,12 +498,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="38" customWidth="1"/>
+    <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
-    <col min="3" max="3" width="26" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
     <col min="5" max="5" width="21" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="8" width="50" customWidth="1"/>
@@ -557,6 +587,58 @@
         <v>22</v>
       </c>
     </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" t="s">
+        <v>31</v>
+      </c>
+      <c r="H5" t="s">
+        <v>32</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>